<commit_message>
Update Game Store pages and logo
</commit_message>
<xml_diff>
--- a/docs/project/Gantt_Final _Final.xlsx
+++ b/docs/project/Gantt_Final _Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\2emeSemestre\M431\Projet-Final\docs\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB1AC208-100D-4690-A0E4-BCDF7D375CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E3F678-D361-4F54-88C1-61AC0E62C20B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt visuel" sheetId="1" r:id="rId1"/>
@@ -388,7 +388,7 @@
     <t>1h30</t>
   </si>
   <si>
-    <t>Game Store - Gantt visuel - Finale</t>
+    <t>Game Store - Gantt visuel - Finale_Finale</t>
   </si>
 </sst>
 </file>
@@ -810,6 +810,9 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -817,9 +820,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1007,55 +1007,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="42" t="s">
+      <c r="G1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="42" t="s">
+      <c r="I1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="42" t="s">
+      <c r="J1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="42" t="s">
+      <c r="K1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="42" t="s">
+      <c r="L1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="M1" s="42" t="s">
+      <c r="M1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="42" t="s">
+      <c r="N1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="O1" s="42" t="s">
+      <c r="O1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="P1" s="42" t="s">
+      <c r="P1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="Q1" s="42" t="s">
+      <c r="Q1" s="43" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1075,10 +1075,10 @@
       <c r="Q2" s="20"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="45" t="s">
         <v>1</v>
       </c>
       <c r="D3" s="8"/>
@@ -2152,8 +2152,8 @@
       <c r="I44" s="24"/>
       <c r="J44" s="24"/>
       <c r="K44" s="24"/>
-      <c r="L44" s="45"/>
-      <c r="M44" s="45"/>
+      <c r="L44" s="42"/>
+      <c r="M44" s="42"/>
       <c r="N44" s="24"/>
       <c r="O44" s="24"/>
       <c r="P44" s="24"/>
@@ -2179,8 +2179,8 @@
       <c r="I45" s="26"/>
       <c r="J45" s="26"/>
       <c r="K45" s="26"/>
-      <c r="L45" s="45"/>
-      <c r="M45" s="45"/>
+      <c r="L45" s="42"/>
+      <c r="M45" s="42"/>
       <c r="N45" s="26"/>
       <c r="O45" s="26"/>
       <c r="P45" s="26"/>
@@ -2206,8 +2206,8 @@
       <c r="I46" s="24"/>
       <c r="J46" s="24"/>
       <c r="K46" s="24"/>
-      <c r="L46" s="45"/>
-      <c r="M46" s="45"/>
+      <c r="L46" s="42"/>
+      <c r="M46" s="42"/>
       <c r="N46" s="24"/>
       <c r="O46" s="24"/>
       <c r="P46" s="24"/>
@@ -2255,8 +2255,8 @@
       <c r="J48" s="24"/>
       <c r="K48" s="24"/>
       <c r="L48" s="24"/>
-      <c r="M48" s="45"/>
-      <c r="N48" s="45"/>
+      <c r="M48" s="42"/>
+      <c r="N48" s="42"/>
       <c r="O48" s="24"/>
       <c r="P48" s="24"/>
       <c r="Q48" s="25"/>
@@ -2303,9 +2303,9 @@
       <c r="J50" s="24"/>
       <c r="K50" s="24"/>
       <c r="L50" s="24"/>
-      <c r="M50" s="45"/>
-      <c r="N50" s="45"/>
-      <c r="O50" s="45"/>
+      <c r="M50" s="42"/>
+      <c r="N50" s="42"/>
+      <c r="O50" s="42"/>
       <c r="P50" s="24"/>
       <c r="Q50" s="25"/>
     </row>
@@ -2352,8 +2352,8 @@
       <c r="K52" s="24"/>
       <c r="L52" s="24"/>
       <c r="M52" s="24"/>
-      <c r="N52" s="45"/>
-      <c r="O52" s="45"/>
+      <c r="N52" s="42"/>
+      <c r="O52" s="42"/>
       <c r="P52" s="24"/>
       <c r="Q52" s="25"/>
     </row>
@@ -2401,8 +2401,8 @@
       <c r="L54" s="24"/>
       <c r="M54" s="24"/>
       <c r="N54" s="24"/>
-      <c r="O54" s="45"/>
-      <c r="P54" s="45"/>
+      <c r="O54" s="42"/>
+      <c r="P54" s="42"/>
       <c r="Q54" s="25"/>
     </row>
     <row r="55" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2429,7 +2429,7 @@
       <c r="M55" s="26"/>
       <c r="N55" s="26"/>
       <c r="O55" s="26"/>
-      <c r="P55" s="45"/>
+      <c r="P55" s="42"/>
       <c r="Q55" s="27"/>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>